<commit_message>
fix: make coordinate provenance reproducible
</commit_message>
<xml_diff>
--- a/dist/xlsx/province-capitals.xlsx
+++ b/dist/xlsx/province-capitals.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:H32"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,6 +418,12 @@
       <c r="F1" t="str">
         <v>source_id</v>
       </c>
+      <c r="G1" t="str">
+        <v>source_feature_id</v>
+      </c>
+      <c r="H1" t="str">
+        <v>source_name</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -438,6 +444,12 @@
       <c r="F2" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G2" t="str">
+        <v>143127</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Arāk</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -458,6 +470,12 @@
       <c r="F3" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G3" t="str">
+        <v>118743</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Rasht</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -478,6 +496,12 @@
       <c r="F4" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G4" t="str">
+        <v>116996</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Sari</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -498,6 +522,12 @@
       <c r="F5" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G5" t="str">
+        <v>113646</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Tabriz</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -518,6 +548,12 @@
       <c r="F6" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G6" t="str">
+        <v>121801</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Orūmīyeh</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -538,6 +574,12 @@
       <c r="F7" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G7" t="str">
+        <v>128226</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Kermanshah</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -558,6 +600,12 @@
       <c r="F8" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G8" t="str">
+        <v>144448</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Ahvaz</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -578,6 +626,12 @@
       <c r="F9" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G9" t="str">
+        <v>115019</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Shiraz</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -598,6 +652,12 @@
       <c r="F10" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G10" t="str">
+        <v>128234</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Kerman</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -618,6 +678,12 @@
       <c r="F11" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G11" t="str">
+        <v>124665</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Mashhad</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -638,6 +704,12 @@
       <c r="F12" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G12" t="str">
+        <v>418863</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Isfahan</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -658,6 +730,12 @@
       <c r="F13" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G13" t="str">
+        <v>1159301</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Zahedan</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -678,6 +756,12 @@
       <c r="F14" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G14" t="str">
+        <v>117574</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Sanandaj</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -698,6 +782,12 @@
       <c r="F15" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G15" t="str">
+        <v>132144</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Hamadān</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -718,6 +808,12 @@
       <c r="F16" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G16" t="str">
+        <v>115770</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Shahr-e Kord</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -738,6 +834,12 @@
       <c r="F17" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G17" t="str">
+        <v>127349</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Khorramabad</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -758,6 +860,12 @@
       <c r="F18" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G18" t="str">
+        <v>130802</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Īlām</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -778,6 +886,12 @@
       <c r="F19" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G19" t="str">
+        <v>66093</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Yasuj</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -798,6 +912,12 @@
       <c r="F20" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G20" t="str">
+        <v>139817</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Bushehr</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -818,6 +938,12 @@
       <c r="F21" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G21" t="str">
+        <v>111453</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Zanjan</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -838,6 +964,12 @@
       <c r="F22" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G22" t="str">
+        <v>116402</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Semnan</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -858,6 +990,12 @@
       <c r="F23" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G23" t="str">
+        <v>111822</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Yazd</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -878,6 +1016,12 @@
       <c r="F24" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G24" t="str">
+        <v>141681</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Bandar Abbas</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -898,6 +1042,12 @@
       <c r="F25" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G25" t="str">
+        <v>6683528</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Tehrān</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -918,6 +1068,12 @@
       <c r="F26" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G26" t="str">
+        <v>143083</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Ardabīl</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -938,6 +1094,12 @@
       <c r="F27" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G27" t="str">
+        <v>119208</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Qom</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -958,6 +1120,12 @@
       <c r="F28" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G28" t="str">
+        <v>119505</v>
+      </c>
+      <c r="H28" t="str">
+        <v>Qazvin</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -978,6 +1146,12 @@
       <c r="F29" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G29" t="str">
+        <v>132892</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Gorgān</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -998,6 +1172,12 @@
       <c r="F30" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G30" t="str">
+        <v>140380</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Bojnūrd</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -1018,6 +1198,12 @@
       <c r="F31" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G31" t="str">
+        <v>140463</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Bīrjand</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -1038,10 +1224,16 @@
       <c r="F32" t="str">
         <v>geonames-iran-2026-09-19</v>
       </c>
+      <c r="G32" t="str">
+        <v>128747</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Karaj</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H32"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>